<commit_message>
Add supplied author affiliations and remove visible commit hashes
</commit_message>
<xml_diff>
--- a/manuscript/annals/concise-report/Supporting_Tables.xlsx
+++ b/manuscript/annals/concise-report/Supporting_Tables.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="1" r:id="R068b7db3614a40ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2" sheetId="2" r:id="Rba0cb703245f4408"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3" sheetId="3" r:id="Re780690847204ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S4" sheetId="4" r:id="R578ed10676304931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="1" r:id="R25da346ecc254780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2" sheetId="2" r:id="R87dd2dbe42864994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3" sheetId="3" r:id="Rcdefb3c8dfeb40fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S4" sheetId="4" r:id="Rbecb2f92d7bd4dc0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -435,7 +435,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2" t="str">
-        <x:v>Source: PhytoScope Supporting Information, evidence snapshot 159ae0f79bd3681afc6c914db282c515190a3888; https://github.com/omixcore/phytoscope</x:v>
+        <x:v>Source: PhytoScope Supporting Information; https://github.com/omixcore/phytoscope</x:v>
       </x:c>
       <x:c r="B13" s="2"/>
       <x:c r="C13" s="2"/>
@@ -622,7 +622,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="2" t="str">
-        <x:v>Source: PhytoScope Supporting Information, evidence snapshot 159ae0f79bd3681afc6c914db282c515190a3888; https://github.com/omixcore/phytoscope</x:v>
+        <x:v>Source: PhytoScope Supporting Information; https://github.com/omixcore/phytoscope</x:v>
       </x:c>
       <x:c r="B15" s="2"/>
       <x:c r="C15" s="2"/>
@@ -767,7 +767,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="str">
-        <x:v>Source: PhytoScope Supporting Information, evidence snapshot 159ae0f79bd3681afc6c914db282c515190a3888; https://github.com/omixcore/phytoscope</x:v>
+        <x:v>Source: PhytoScope Supporting Information; https://github.com/omixcore/phytoscope</x:v>
       </x:c>
       <x:c r="B18" s="2"/>
     </x:row>
@@ -908,7 +908,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="2" t="str">
-        <x:v>Source: PhytoScope Supporting Information, evidence snapshot 159ae0f79bd3681afc6c914db282c515190a3888; https://github.com/omixcore/phytoscope</x:v>
+        <x:v>Source: PhytoScope Supporting Information; https://github.com/omixcore/phytoscope</x:v>
       </x:c>
       <x:c r="B12" s="2"/>
       <x:c r="C12" s="2"/>

</xml_diff>